<commit_message>
Deploy: Update Документ “perechen-smsp” +1 c8b3a2e0bf54d8a8be613713b8493beb8796f179
</commit_message>
<xml_diff>
--- a/uploads/perechen-zakupok-smsp.xlsx
+++ b/uploads/perechen-zakupok-smsp.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\moscollector.local\docs\ООЗ\ЗАКУПКИ 2026\ПЕРЕЧЕНЬ ЗАКУПОК У СМСП\Корректировка 4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\moscollector.local\docs\ООЗ\ЗАКУПКИ 2026\ПЕРЕЧЕНЬ ЗАКУПОК У СМСП\Корректировка 5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA9620E1-932E-4FFA-A297-C890D603DAA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B80C5173-FCE0-49BD-AB84-A0288316BAA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="750" yWindow="885" windowWidth="25350" windowHeight="13995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Лист1!$A$8:$C$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Лист1!$A$1:$C$286</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Лист1!$A$1:$C$291</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="553">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="561">
   <si>
     <t>ОКПД 2</t>
   </si>
@@ -1714,13 +1714,37 @@
     <t>Пленки прочие пластмассовые пористые</t>
   </si>
   <si>
-    <t xml:space="preserve">Первый заместитель генерального директора              </t>
-  </si>
-  <si>
-    <t xml:space="preserve">                                                                      М.В. Епифанцев</t>
-  </si>
-  <si>
-    <t>к приказу от 14.05.2026 № 186</t>
+    <t xml:space="preserve">31.02.10.120 </t>
+  </si>
+  <si>
+    <t>Шкафы кухонные</t>
+  </si>
+  <si>
+    <t>31.02.10.190</t>
+  </si>
+  <si>
+    <t>Мебель кухонная прочая</t>
+  </si>
+  <si>
+    <t>31.09.12.131</t>
+  </si>
+  <si>
+    <t>Столы обеденные деревянные для столовой и гостиной</t>
+  </si>
+  <si>
+    <t>81.22.12.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Услуги по чистке и уборке специализированные </t>
+  </si>
+  <si>
+    <t>61.20.50.110</t>
+  </si>
+  <si>
+    <t>Услуги связи для целей эфирного вещания</t>
+  </si>
+  <si>
+    <t>к приказу от 16.06.2026 № 237</t>
   </si>
 </sst>
 </file>
@@ -1855,7 +1879,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1963,6 +1987,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2315,7 +2343,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J284"/>
+  <dimension ref="A1:J289"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="12" customWidth="1"/>
@@ -2332,7 +2360,7 @@
     </row>
     <row r="2" spans="1:4" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C2" s="39" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2342,21 +2370,21 @@
       <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:4" ht="3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="43" t="s">
         <v>335</v>
       </c>
-      <c r="B5" s="41"/>
-      <c r="C5" s="41"/>
+      <c r="B5" s="43"/>
+      <c r="C5" s="43"/>
     </row>
     <row r="6" spans="1:4" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="41"/>
-      <c r="B6" s="41"/>
-      <c r="C6" s="41"/>
+      <c r="A6" s="43"/>
+      <c r="B6" s="43"/>
+      <c r="C6" s="43"/>
     </row>
     <row r="7" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="42"/>
-      <c r="B7" s="42"/>
-      <c r="C7" s="42"/>
+      <c r="A7" s="44"/>
+      <c r="B7" s="44"/>
+      <c r="C7" s="44"/>
     </row>
     <row r="8" spans="1:4" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
@@ -4710,7 +4738,7 @@
     </row>
     <row r="204" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="5">
-        <f t="shared" ref="A204:A267" si="3">A203+1</f>
+        <f t="shared" ref="A204:A213" si="3">A203+1</f>
         <v>196</v>
       </c>
       <c r="B204" s="5" t="s">
@@ -4828,842 +4856,824 @@
         <v>538</v>
       </c>
     </row>
-    <row r="214" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A214" s="5">
-        <f t="shared" si="3"/>
         <v>206</v>
       </c>
       <c r="B214" s="5" t="s">
+        <v>550</v>
+      </c>
+      <c r="C214" s="42" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A215" s="5">
+        <v>207</v>
+      </c>
+      <c r="B215" s="5" t="s">
+        <v>552</v>
+      </c>
+      <c r="C215" s="7" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A216" s="5">
+        <v>208</v>
+      </c>
+      <c r="B216" s="5" t="s">
         <v>419</v>
       </c>
-      <c r="C214" s="7" t="s">
+      <c r="C216" s="7" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="215" spans="1:3" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A215" s="5">
-        <f t="shared" si="3"/>
-        <v>207</v>
-      </c>
-      <c r="B215" s="24" t="s">
+    <row r="217" spans="1:3" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A217" s="5">
+        <v>209</v>
+      </c>
+      <c r="B217" s="24" t="s">
         <v>455</v>
       </c>
-      <c r="C215" s="9" t="s">
+      <c r="C217" s="9" t="s">
         <v>456</v>
       </c>
     </row>
-    <row r="216" spans="1:3" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A216" s="5">
-        <f t="shared" si="3"/>
-        <v>208</v>
-      </c>
-      <c r="B216" s="24" t="s">
+    <row r="218" spans="1:3" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A218" s="5">
+        <v>210</v>
+      </c>
+      <c r="B218" s="24" t="s">
         <v>523</v>
       </c>
-      <c r="C216" s="9" t="s">
+      <c r="C218" s="9" t="s">
         <v>524</v>
       </c>
     </row>
-    <row r="217" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A217" s="5">
-        <f t="shared" si="3"/>
-        <v>209</v>
-      </c>
-      <c r="B217" s="5" t="s">
+    <row r="219" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A219" s="5">
+        <v>211</v>
+      </c>
+      <c r="B219" s="5" t="s">
+        <v>554</v>
+      </c>
+      <c r="C219" s="7" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A220" s="5">
+        <v>212</v>
+      </c>
+      <c r="B220" s="5" t="s">
         <v>421</v>
       </c>
-      <c r="C217" s="7" t="s">
+      <c r="C220" s="7" t="s">
         <v>422</v>
       </c>
     </row>
-    <row r="218" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A218" s="5">
-        <f t="shared" si="3"/>
-        <v>210</v>
-      </c>
-      <c r="B218" s="5" t="s">
+    <row r="221" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A221" s="5">
+        <v>213</v>
+      </c>
+      <c r="B221" s="5" t="s">
         <v>525</v>
       </c>
-      <c r="C218" s="7" t="s">
+      <c r="C221" s="7" t="s">
         <v>526</v>
       </c>
     </row>
-    <row r="219" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A219" s="5">
-        <f t="shared" si="3"/>
-        <v>211</v>
-      </c>
-      <c r="B219" s="5" t="s">
+    <row r="222" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A222" s="5">
+        <v>214</v>
+      </c>
+      <c r="B222" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="C219" s="7" t="s">
+      <c r="C222" s="7" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A220" s="5">
-        <f t="shared" si="3"/>
-        <v>212</v>
-      </c>
-      <c r="B220" s="5" t="s">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A223" s="5">
+        <v>215</v>
+      </c>
+      <c r="B223" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="C220" s="7" t="s">
+      <c r="C223" s="7" t="s">
         <v>334</v>
-      </c>
-    </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A221" s="5">
-        <f t="shared" si="3"/>
-        <v>213</v>
-      </c>
-      <c r="B221" s="6" t="s">
-        <v>318</v>
-      </c>
-      <c r="C221" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A222" s="5">
-        <f t="shared" si="3"/>
-        <v>214</v>
-      </c>
-      <c r="B222" s="6" t="s">
-        <v>320</v>
-      </c>
-      <c r="C222" s="7" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="223" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A223" s="5">
-        <f t="shared" si="3"/>
-        <v>215</v>
-      </c>
-      <c r="B223" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="C223" s="9" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" s="5">
-        <f t="shared" si="3"/>
         <v>216</v>
       </c>
       <c r="B224" s="6" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="C224" s="7" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="225" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" s="5">
-        <f t="shared" si="3"/>
         <v>217</v>
       </c>
       <c r="B225" s="6" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="C225" s="7" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A226" s="5">
-        <f t="shared" si="3"/>
         <v>218</v>
       </c>
-      <c r="B226" s="6" t="s">
-        <v>326</v>
-      </c>
-      <c r="C226" s="7" t="s">
-        <v>327</v>
+      <c r="B226" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C226" s="9" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227" s="5">
-        <f t="shared" si="3"/>
         <v>219</v>
       </c>
       <c r="B227" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="C227" s="7" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A228" s="5">
+        <v>220</v>
+      </c>
+      <c r="B228" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="C228" s="7" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A229" s="5">
+        <v>221</v>
+      </c>
+      <c r="B229" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C229" s="7" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A230" s="5">
+        <v>222</v>
+      </c>
+      <c r="B230" s="6" t="s">
         <v>328</v>
       </c>
-      <c r="C227" s="7" t="s">
+      <c r="C230" s="7" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="228" spans="1:3" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A228" s="5">
-        <f t="shared" si="3"/>
-        <v>220</v>
-      </c>
-      <c r="B228" s="5" t="s">
+    <row r="231" spans="1:3" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A231" s="5">
+        <v>223</v>
+      </c>
+      <c r="B231" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="C228" s="7" t="s">
+      <c r="C231" s="7" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="229" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A229" s="5">
-        <f t="shared" si="3"/>
-        <v>221</v>
-      </c>
-      <c r="B229" s="5" t="s">
+    <row r="232" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A232" s="5">
+        <v>224</v>
+      </c>
+      <c r="B232" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C229" s="7" t="s">
+      <c r="C232" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="230" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A230" s="5">
-        <f t="shared" si="3"/>
-        <v>222</v>
-      </c>
-      <c r="B230" s="5" t="s">
+    <row r="233" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A233" s="5">
+        <v>225</v>
+      </c>
+      <c r="B233" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="C230" s="7" t="s">
+      <c r="C233" s="7" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="231" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A231" s="5">
-        <f t="shared" si="3"/>
-        <v>223</v>
-      </c>
-      <c r="B231" s="5" t="s">
+    <row r="234" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A234" s="5">
+        <v>226</v>
+      </c>
+      <c r="B234" s="5" t="s">
         <v>387</v>
       </c>
-      <c r="C231" s="7" t="s">
+      <c r="C234" s="7" t="s">
         <v>388</v>
-      </c>
-    </row>
-    <row r="232" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A232" s="5">
-        <f t="shared" si="3"/>
-        <v>224</v>
-      </c>
-      <c r="B232" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="C232" s="7" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="233" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A233" s="5">
-        <f t="shared" si="3"/>
-        <v>225</v>
-      </c>
-      <c r="B233" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="C233" s="7" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="234" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A234" s="5">
-        <f t="shared" si="3"/>
-        <v>226</v>
-      </c>
-      <c r="B234" s="8" t="s">
-        <v>382</v>
-      </c>
-      <c r="C234" s="7" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="235" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A235" s="5">
-        <f t="shared" si="3"/>
         <v>227</v>
       </c>
       <c r="B235" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C235" s="7" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="236" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A236" s="5">
+        <v>228</v>
+      </c>
+      <c r="B236" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="C236" s="7" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A237" s="5">
+        <v>229</v>
+      </c>
+      <c r="B237" s="8" t="s">
+        <v>382</v>
+      </c>
+      <c r="C237" s="7" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A238" s="5">
+        <v>230</v>
+      </c>
+      <c r="B238" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="C235" s="7" t="s">
+      <c r="C238" s="7" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="236" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A236" s="5">
-        <f t="shared" si="3"/>
-        <v>228</v>
-      </c>
-      <c r="B236" s="5" t="s">
+    <row r="239" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A239" s="5">
+        <v>231</v>
+      </c>
+      <c r="B239" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="C236" s="7" t="s">
+      <c r="C239" s="7" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="237" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A237" s="5">
-        <f t="shared" si="3"/>
-        <v>229</v>
-      </c>
-      <c r="B237" s="8" t="s">
+    <row r="240" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A240" s="5">
+        <v>232</v>
+      </c>
+      <c r="B240" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="C237" s="7" t="s">
+      <c r="C240" s="7" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="238" spans="1:3" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A238" s="5">
-        <f t="shared" si="3"/>
-        <v>230</v>
-      </c>
-      <c r="B238" s="8" t="s">
+    <row r="241" spans="1:3" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A241" s="5">
+        <v>233</v>
+      </c>
+      <c r="B241" s="8" t="s">
         <v>384</v>
       </c>
-      <c r="C238" s="7" t="s">
+      <c r="C241" s="7" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="239" spans="1:3" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A239" s="5">
-        <f t="shared" si="3"/>
-        <v>231</v>
-      </c>
-      <c r="B239" s="8" t="s">
+    <row r="242" spans="1:3" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A242" s="5">
+        <v>234</v>
+      </c>
+      <c r="B242" s="8" t="s">
         <v>360</v>
       </c>
-      <c r="C239" s="7" t="s">
+      <c r="C242" s="7" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="240" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A240" s="5">
-        <f t="shared" si="3"/>
-        <v>232</v>
-      </c>
-      <c r="B240" s="8" t="s">
+    <row r="243" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A243" s="5">
+        <v>235</v>
+      </c>
+      <c r="B243" s="8" t="s">
         <v>409</v>
       </c>
-      <c r="C240" s="7" t="s">
+      <c r="C243" s="7" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="241" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A241" s="5">
-        <f t="shared" si="3"/>
-        <v>233</v>
-      </c>
-      <c r="B241" s="8" t="s">
+    <row r="244" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A244" s="5">
+        <v>236</v>
+      </c>
+      <c r="B244" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C241" s="7" t="s">
+      <c r="C244" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="242" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A242" s="5">
-        <f t="shared" si="3"/>
-        <v>234</v>
-      </c>
-      <c r="B242" s="8" t="s">
+    <row r="245" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A245" s="5">
+        <v>237</v>
+      </c>
+      <c r="B245" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C242" s="7" t="s">
+      <c r="C245" s="7" t="s">
         <v>149</v>
-      </c>
-    </row>
-    <row r="243" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A243" s="5">
-        <f t="shared" si="3"/>
-        <v>235</v>
-      </c>
-      <c r="B243" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="C243" s="7" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A244" s="5">
-        <f t="shared" si="3"/>
-        <v>236</v>
-      </c>
-      <c r="B244" s="5" t="s">
-        <v>358</v>
-      </c>
-      <c r="C244" s="7" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="245" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A245" s="5">
-        <f t="shared" si="3"/>
-        <v>237</v>
-      </c>
-      <c r="B245" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="C245" s="7" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="246" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A246" s="5">
-        <f t="shared" si="3"/>
         <v>238</v>
       </c>
       <c r="B246" s="5" t="s">
-        <v>246</v>
+        <v>153</v>
       </c>
       <c r="C246" s="7" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="247" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" s="5">
-        <f t="shared" si="3"/>
         <v>239</v>
       </c>
-      <c r="B247" s="8" t="s">
-        <v>10</v>
+      <c r="B247" s="5" t="s">
+        <v>358</v>
       </c>
       <c r="C247" s="7" t="s">
-        <v>11</v>
+        <v>359</v>
       </c>
     </row>
     <row r="248" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A248" s="5">
-        <f t="shared" si="3"/>
         <v>240</v>
       </c>
-      <c r="B248" s="8" t="s">
+      <c r="B248" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="C248" s="7" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A249" s="5">
+        <v>241</v>
+      </c>
+      <c r="B249" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="C249" s="7" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="250" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A250" s="5">
+        <v>242</v>
+      </c>
+      <c r="B250" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C250" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="251" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A251" s="5">
+        <v>243</v>
+      </c>
+      <c r="B251" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C248" s="7" t="s">
+      <c r="C251" s="7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A249" s="5">
-        <f t="shared" si="3"/>
-        <v>241</v>
-      </c>
-      <c r="B249" s="8" t="s">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A252" s="5">
+        <v>244</v>
+      </c>
+      <c r="B252" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="C249" s="7" t="s">
+      <c r="C252" s="7" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A250" s="5">
-        <f t="shared" si="3"/>
-        <v>242</v>
-      </c>
-      <c r="B250" s="8" t="s">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A253" s="5">
+        <v>245</v>
+      </c>
+      <c r="B253" s="8" t="s">
         <v>386</v>
       </c>
-      <c r="C250" s="7" t="s">
+      <c r="C253" s="7" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A251" s="5">
-        <f t="shared" si="3"/>
-        <v>243</v>
-      </c>
-      <c r="B251" s="8" t="s">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A254" s="5">
+        <v>246</v>
+      </c>
+      <c r="B254" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="C251" s="7" t="s">
+      <c r="C254" s="7" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="252" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A252" s="5">
-        <f t="shared" si="3"/>
-        <v>244</v>
-      </c>
-      <c r="B252" s="8" t="s">
+    <row r="255" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A255" s="5">
+        <v>247</v>
+      </c>
+      <c r="B255" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="C252" s="9" t="s">
+      <c r="C255" s="9" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="253" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A253" s="5">
-        <f t="shared" si="3"/>
-        <v>245</v>
-      </c>
-      <c r="B253" s="8" t="s">
+    <row r="256" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A256" s="5">
+        <v>248</v>
+      </c>
+      <c r="B256" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="C253" s="9" t="s">
+      <c r="C256" s="9" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="254" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A254" s="5">
-        <f t="shared" si="3"/>
-        <v>246</v>
-      </c>
-      <c r="B254" s="8" t="s">
+    <row r="257" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A257" s="5">
+        <v>249</v>
+      </c>
+      <c r="B257" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="C254" s="9" t="s">
+      <c r="C257" s="9" t="s">
         <v>134</v>
-      </c>
-    </row>
-    <row r="255" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A255" s="5">
-        <f t="shared" si="3"/>
-        <v>247</v>
-      </c>
-      <c r="B255" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="C255" s="9" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="256" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A256" s="5">
-        <f t="shared" si="3"/>
-        <v>248</v>
-      </c>
-      <c r="B256" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="C256" s="9" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A257" s="5">
-        <f t="shared" si="3"/>
-        <v>249</v>
-      </c>
-      <c r="B257" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="C257" s="9" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="258" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A258" s="5">
-        <f t="shared" si="3"/>
         <v>250</v>
       </c>
       <c r="B258" s="8" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="C258" s="9" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="259" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A259" s="5">
-        <f t="shared" si="3"/>
         <v>251</v>
       </c>
-      <c r="B259" s="8" t="s">
-        <v>143</v>
+      <c r="B259" s="5" t="s">
+        <v>137</v>
       </c>
       <c r="C259" s="9" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="260" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" s="5">
-        <f t="shared" si="3"/>
         <v>252</v>
       </c>
       <c r="B260" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="C260" s="7" t="s">
-        <v>4</v>
+        <v>139</v>
+      </c>
+      <c r="C260" s="9" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="261" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A261" s="5">
-        <f t="shared" si="3"/>
         <v>253</v>
       </c>
       <c r="B261" s="8" t="s">
-        <v>221</v>
-      </c>
-      <c r="C261" s="7" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.3">
+        <v>141</v>
+      </c>
+      <c r="C261" s="9" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" s="5">
-        <f t="shared" si="3"/>
         <v>254</v>
       </c>
-      <c r="B262" s="31" t="s">
-        <v>527</v>
-      </c>
-      <c r="C262" s="7" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B262" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="C262" s="9" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A263" s="5">
-        <f t="shared" si="3"/>
         <v>255</v>
       </c>
       <c r="B263" s="8" t="s">
-        <v>354</v>
+        <v>2</v>
       </c>
       <c r="C263" s="7" t="s">
-        <v>355</v>
+        <v>4</v>
       </c>
     </row>
     <row r="264" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A264" s="5">
-        <f t="shared" si="3"/>
         <v>256</v>
       </c>
       <c r="B264" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="C264" s="7" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A265" s="5">
+        <v>257</v>
+      </c>
+      <c r="B265" s="31" t="s">
+        <v>527</v>
+      </c>
+      <c r="C265" s="7" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A266" s="5">
+        <v>258</v>
+      </c>
+      <c r="B266" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="C266" s="7" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A267" s="5">
+        <v>259</v>
+      </c>
+      <c r="B267" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="C264" s="7" t="s">
+      <c r="C267" s="7" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="265" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A265" s="5">
-        <f t="shared" si="3"/>
-        <v>257</v>
-      </c>
-      <c r="B265" s="8" t="s">
+    <row r="268" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A268" s="5">
+        <v>260</v>
+      </c>
+      <c r="B268" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C265" s="7" t="s">
+      <c r="C268" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="266" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A266" s="5">
-        <f t="shared" si="3"/>
-        <v>258</v>
-      </c>
-      <c r="B266" s="8" t="s">
+    <row r="269" spans="1:3" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A269" s="24">
+        <v>261</v>
+      </c>
+      <c r="B269" s="41" t="s">
+        <v>558</v>
+      </c>
+      <c r="C269" s="9" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="270" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A270" s="5">
+        <v>262</v>
+      </c>
+      <c r="B270" s="8" t="s">
         <v>356</v>
       </c>
-      <c r="C266" s="7" t="s">
+      <c r="C270" s="7" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="267" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A267" s="5">
-        <f t="shared" si="3"/>
-        <v>259</v>
-      </c>
-      <c r="B267" s="8" t="s">
+    <row r="271" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A271" s="5">
+        <v>263</v>
+      </c>
+      <c r="B271" s="8" t="s">
         <v>453</v>
       </c>
-      <c r="C267" s="7" t="s">
+      <c r="C271" s="7" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="268" spans="1:3" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A268" s="5">
-        <f t="shared" ref="A268:A281" si="4">A267+1</f>
-        <v>260</v>
-      </c>
-      <c r="B268" s="8" t="s">
+    <row r="272" spans="1:3" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A272" s="5">
+        <v>264</v>
+      </c>
+      <c r="B272" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C268" s="7" t="s">
+      <c r="C272" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="269" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A269" s="5">
-        <f t="shared" si="4"/>
-        <v>261</v>
-      </c>
-      <c r="B269" s="29" t="s">
+    <row r="273" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A273" s="5">
+        <v>265</v>
+      </c>
+      <c r="B273" s="29" t="s">
         <v>489</v>
       </c>
-      <c r="C269" s="28" t="s">
+      <c r="C273" s="28" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="270" spans="1:3" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A270" s="5">
-        <f t="shared" si="4"/>
-        <v>262</v>
-      </c>
-      <c r="B270" s="8" t="s">
+    <row r="274" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A274" s="5">
+        <v>266</v>
+      </c>
+      <c r="B274" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C270" s="7" t="s">
+      <c r="C274" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="271" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A271" s="5">
-        <f t="shared" si="4"/>
-        <v>263</v>
-      </c>
-      <c r="B271" s="5" t="s">
+    <row r="275" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A275" s="5">
+        <v>267</v>
+      </c>
+      <c r="B275" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="C271" s="7" t="s">
+      <c r="C275" s="7" t="s">
         <v>151</v>
-      </c>
-    </row>
-    <row r="272" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A272" s="5">
-        <f t="shared" si="4"/>
-        <v>264</v>
-      </c>
-      <c r="B272" s="6" t="s">
-        <v>330</v>
-      </c>
-      <c r="C272" s="7" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="273" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A273" s="5">
-        <f t="shared" si="4"/>
-        <v>265</v>
-      </c>
-      <c r="B273" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="C273" s="7" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="274" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A274" s="5">
-        <f t="shared" si="4"/>
-        <v>266</v>
-      </c>
-      <c r="B274" s="5" t="s">
-        <v>423</v>
-      </c>
-      <c r="C274" s="7" t="s">
-        <v>424</v>
-      </c>
-      <c r="J274" s="21"/>
-    </row>
-    <row r="275" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A275" s="5">
-        <f t="shared" si="4"/>
-        <v>267</v>
-      </c>
-      <c r="B275" s="5" t="s">
-        <v>239</v>
-      </c>
-      <c r="C275" s="7" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="276" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A276" s="5">
-        <f t="shared" si="4"/>
         <v>268</v>
       </c>
-      <c r="B276" s="5" t="s">
-        <v>200</v>
+      <c r="B276" s="6" t="s">
+        <v>330</v>
       </c>
       <c r="C276" s="7" t="s">
-        <v>201</v>
+        <v>331</v>
       </c>
     </row>
     <row r="277" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A277" s="5">
-        <f t="shared" si="4"/>
         <v>269</v>
       </c>
       <c r="B277" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="C277" s="7" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="278" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A278" s="5">
+        <v>270</v>
+      </c>
+      <c r="B278" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="C278" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="J278" s="21"/>
+    </row>
+    <row r="279" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A279" s="5">
+        <v>271</v>
+      </c>
+      <c r="B279" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="C279" s="7" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="280" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A280" s="5">
+        <v>272</v>
+      </c>
+      <c r="B280" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="C280" s="7" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="281" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A281" s="5">
+        <v>273</v>
+      </c>
+      <c r="B281" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C277" s="7" t="s">
+      <c r="C281" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="278" spans="1:10" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A278" s="5">
-        <f t="shared" si="4"/>
-        <v>270</v>
-      </c>
-      <c r="B278" s="5" t="s">
+    <row r="282" spans="1:10" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A282" s="5">
+        <v>274</v>
+      </c>
+      <c r="B282" s="5" t="s">
         <v>437</v>
       </c>
-      <c r="C278" s="22" t="s">
+      <c r="C282" s="22" t="s">
         <v>438</v>
       </c>
     </row>
-    <row r="279" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A279" s="5">
-        <f t="shared" si="4"/>
-        <v>271</v>
-      </c>
-      <c r="B279" s="5" t="s">
+    <row r="283" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A283" s="5">
+        <v>275</v>
+      </c>
+      <c r="B283" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="C279" s="7" t="s">
+      <c r="C283" s="7" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="280" spans="1:10" s="25" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A280" s="5">
-        <f t="shared" si="4"/>
-        <v>272</v>
-      </c>
-      <c r="B280" s="5" t="s">
+    <row r="284" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A284" s="5">
+        <v>276</v>
+      </c>
+      <c r="B284" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="C284" s="23" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="285" spans="1:10" s="25" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A285" s="5">
+        <v>277</v>
+      </c>
+      <c r="B285" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C280" s="23" t="s">
+      <c r="C285" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="281" spans="1:10" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A281" s="5">
-        <f t="shared" si="4"/>
-        <v>273</v>
-      </c>
-      <c r="B281" s="5" t="s">
+    <row r="286" spans="1:10" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A286" s="5">
+        <v>278</v>
+      </c>
+      <c r="B286" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="C281" s="7" t="s">
+      <c r="C286" s="7" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="282" spans="1:10" ht="15" x14ac:dyDescent="0.25">
-      <c r="A282" s="1"/>
-      <c r="B282" s="1"/>
-      <c r="C282" s="1"/>
-    </row>
-    <row r="284" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A284" s="12" t="s">
-        <v>550</v>
-      </c>
-      <c r="C284" s="40" t="s">
-        <v>551</v>
-      </c>
-      <c r="D284" s="36"/>
-      <c r="E284" s="37"/>
-      <c r="F284" s="37"/>
-      <c r="G284" s="38"/>
-      <c r="H284" s="12"/>
-      <c r="I284" s="12"/>
-      <c r="J284" s="12"/>
+    <row r="287" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="A287" s="1"/>
+      <c r="B287" s="1"/>
+      <c r="C287" s="1"/>
+    </row>
+    <row r="289" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C289" s="40"/>
+      <c r="D289" s="36"/>
+      <c r="E289" s="37"/>
+      <c r="F289" s="37"/>
+      <c r="G289" s="38"/>
+      <c r="H289" s="12"/>
+      <c r="I289" s="12"/>
+      <c r="J289" s="12"/>
     </row>
   </sheetData>
   <autoFilter ref="A8:C8" xr:uid="{00000000-0009-0000-0000-000000000000}">
@@ -5676,10 +5686,6 @@
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="66" fitToHeight="0" orientation="portrait" r:id="rId1"/>
-  <rowBreaks count="2" manualBreakCount="2">
-    <brk id="36" max="2" man="1"/>
-    <brk id="234" max="2" man="1"/>
-  </rowBreaks>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Deploy: Update Документ “perechen-smsp” +1 c06e6e47aa1434710f18e579cf2ebb704479f06a
</commit_message>
<xml_diff>
--- a/uploads/perechen-zakupok-smsp.xlsx
+++ b/uploads/perechen-zakupok-smsp.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\moscollector.local\docs\ООЗ\ЗАКУПКИ 2026\ПЕРЕЧЕНЬ ЗАКУПОК У СМСП\Корректировка 5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\moscollector.local\docs\ООЗ\ЗАКУПКИ 2026\ПЕРЕЧЕНЬ ЗАКУПОК У СМСП\Корректировка 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B80C5173-FCE0-49BD-AB84-A0288316BAA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10BB357F-B802-43C5-B66A-35059ED81561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,9 +19,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Лист1!$A$8:$C$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Лист1!$A$1:$C$291</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Лист1!$A$1:$C$292</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" refMode="R1C1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="561">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="563">
   <si>
     <t>ОКПД 2</t>
   </si>
@@ -1744,14 +1744,20 @@
     <t>Услуги связи для целей эфирного вещания</t>
   </si>
   <si>
-    <t>к приказу от 16.06.2026 № 237</t>
+    <t>82.19.11.000</t>
+  </si>
+  <si>
+    <t>Услуги по размножению документов</t>
+  </si>
+  <si>
+    <t>к приказу от 25.06.2026 № 256</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1802,6 +1808,13 @@
       <family val="1"/>
       <charset val="204"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1817,7 +1830,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1875,11 +1888,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1991,6 +2017,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2343,7 +2376,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J289"/>
+  <dimension ref="A1:J290"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="12" customWidth="1"/>
@@ -2360,7 +2393,7 @@
     </row>
     <row r="2" spans="1:4" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C2" s="39" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2370,21 +2403,21 @@
       <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:4" ht="3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="46" t="s">
         <v>335</v>
       </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="43"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="46"/>
     </row>
     <row r="6" spans="1:4" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="43"/>
-      <c r="B6" s="43"/>
-      <c r="C6" s="43"/>
+      <c r="A6" s="46"/>
+      <c r="B6" s="46"/>
+      <c r="C6" s="46"/>
     </row>
     <row r="7" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="44"/>
-      <c r="B7" s="44"/>
-      <c r="C7" s="44"/>
+      <c r="A7" s="47"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
     </row>
     <row r="8" spans="1:4" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
@@ -5638,42 +5671,53 @@
         <v>557</v>
       </c>
     </row>
-    <row r="285" spans="1:10" s="25" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A285" s="5">
         <v>277</v>
       </c>
-      <c r="B285" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C285" s="23" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="286" spans="1:10" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B285" s="43" t="s">
+        <v>560</v>
+      </c>
+      <c r="C285" s="45" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="286" spans="1:10" s="25" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A286" s="5">
         <v>278</v>
       </c>
-      <c r="B286" s="5" t="s">
+      <c r="B286" s="44" t="s">
+        <v>18</v>
+      </c>
+      <c r="C286" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="287" spans="1:10" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A287" s="5">
+        <v>279</v>
+      </c>
+      <c r="B287" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="C286" s="7" t="s">
+      <c r="C287" s="7" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="287" spans="1:10" ht="15" x14ac:dyDescent="0.25">
-      <c r="A287" s="1"/>
-      <c r="B287" s="1"/>
-      <c r="C287" s="1"/>
-    </row>
-    <row r="289" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C289" s="40"/>
-      <c r="D289" s="36"/>
-      <c r="E289" s="37"/>
-      <c r="F289" s="37"/>
-      <c r="G289" s="38"/>
-      <c r="H289" s="12"/>
-      <c r="I289" s="12"/>
-      <c r="J289" s="12"/>
+    <row r="288" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="A288" s="1"/>
+      <c r="B288" s="1"/>
+      <c r="C288" s="1"/>
+    </row>
+    <row r="290" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C290" s="40"/>
+      <c r="D290" s="36"/>
+      <c r="E290" s="37"/>
+      <c r="F290" s="37"/>
+      <c r="G290" s="38"/>
+      <c r="H290" s="12"/>
+      <c r="I290" s="12"/>
+      <c r="J290" s="12"/>
     </row>
   </sheetData>
   <autoFilter ref="A8:C8" xr:uid="{00000000-0009-0000-0000-000000000000}">

</xml_diff>

<commit_message>
Deploy: Update Документ “perechen-smsp” +1 257f9f67f6d58008e2b262257ae4f849ae1b5a92
</commit_message>
<xml_diff>
--- a/uploads/perechen-zakupok-smsp.xlsx
+++ b/uploads/perechen-zakupok-smsp.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\moscollector.local\docs\ООЗ\ЗАКУПКИ 2026\ПЕРЕЧЕНЬ ЗАКУПОК У СМСП\Корректировка 6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\moscollector.local\docs\ООЗ\ЗАКУПКИ 2026\ПЕРЕЧЕНЬ ЗАКУПОК У СМСП\Корректировка 7\На сайт\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10BB357F-B802-43C5-B66A-35059ED81561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF81034C-F4EE-4B6A-A9DA-6A1F7901BC7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,9 +19,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Лист1!$A$8:$C$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Лист1!$A$1:$C$292</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Лист1!$A$1:$C$291</definedName>
   </definedNames>
-  <calcPr calcId="191029" refMode="R1C1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="566">
   <si>
     <t>ОКПД 2</t>
   </si>
@@ -1750,14 +1750,54 @@
     <t>Услуги по размножению документов</t>
   </si>
   <si>
-    <t>к приказу от 25.06.2026 № 256</t>
+    <t>Моноблоки</t>
+  </si>
+  <si>
+    <t>26.20.15.140</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">к приказу от </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="14"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">  03.08.2026 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve"> № </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="14"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">307  </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">                                                                                               </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1811,6 +1851,13 @@
     <font>
       <sz val="14"/>
       <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="14"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="204"/>
@@ -1905,7 +1952,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2010,9 +2057,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2024,6 +2068,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2376,11 +2427,11 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J290"/>
+  <dimension ref="A1:J291"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="12" customWidth="1"/>
-    <col min="2" max="2" width="42" style="13" customWidth="1"/>
+    <col min="2" max="2" width="48.140625" style="13" customWidth="1"/>
     <col min="3" max="3" width="79.5703125" style="12" customWidth="1"/>
     <col min="4" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -2393,7 +2444,7 @@
     </row>
     <row r="2" spans="1:4" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C2" s="39" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2403,21 +2454,21 @@
       <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:4" ht="3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="48" t="s">
         <v>335</v>
       </c>
-      <c r="B5" s="46"/>
-      <c r="C5" s="46"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="48"/>
     </row>
     <row r="6" spans="1:4" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="46"/>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
+      <c r="A6" s="48"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
     </row>
     <row r="7" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="47"/>
-      <c r="B7" s="47"/>
-      <c r="C7" s="47"/>
+      <c r="A7" s="49"/>
+      <c r="B7" s="49"/>
+      <c r="C7" s="49"/>
     </row>
     <row r="8" spans="1:4" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
@@ -3223,7 +3274,7 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="5">
-        <f t="shared" ref="A75:A139" si="1">A74+1</f>
+        <f t="shared" ref="A75:A140" si="1">A74+1</f>
         <v>67</v>
       </c>
       <c r="B75" s="11" t="s">
@@ -3881,52 +3932,52 @@
         <v>371</v>
       </c>
     </row>
-    <row r="130" spans="1:3" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="5">
+    <row r="130" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="47">
         <f t="shared" si="1"/>
         <v>122</v>
       </c>
-      <c r="B130" s="6" t="s">
+      <c r="B130" s="27" t="s">
+        <v>563</v>
+      </c>
+      <c r="C130" s="28" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="5">
+        <f t="shared" si="1"/>
+        <v>123</v>
+      </c>
+      <c r="B131" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="C130" s="7" t="s">
+      <c r="C131" s="7" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="131" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A131" s="5">
-        <f t="shared" si="1"/>
-        <v>123</v>
-      </c>
-      <c r="B131" s="6" t="s">
+    <row r="132" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A132" s="5">
+        <f t="shared" si="1"/>
+        <v>124</v>
+      </c>
+      <c r="B132" s="6" t="s">
         <v>457</v>
       </c>
-      <c r="C131" s="7" t="s">
+      <c r="C132" s="7" t="s">
         <v>458</v>
       </c>
     </row>
-    <row r="132" spans="1:3" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="5">
-        <f t="shared" si="1"/>
-        <v>124</v>
-      </c>
-      <c r="B132" s="5" t="s">
+    <row r="133" spans="1:3" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A133" s="5">
+        <f t="shared" si="1"/>
+        <v>125</v>
+      </c>
+      <c r="B133" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="C132" s="7" t="s">
+      <c r="C133" s="7" t="s">
         <v>254</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A133" s="5">
-        <f t="shared" si="1"/>
-        <v>125</v>
-      </c>
-      <c r="B133" s="6" t="s">
-        <v>295</v>
-      </c>
-      <c r="C133" s="7" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
@@ -3935,10 +3986,10 @@
         <v>126</v>
       </c>
       <c r="B134" s="6" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C134" s="7" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
@@ -3947,130 +3998,130 @@
         <v>127</v>
       </c>
       <c r="B135" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="C135" s="7" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A136" s="5">
+        <f t="shared" si="1"/>
+        <v>128</v>
+      </c>
+      <c r="B136" s="6" t="s">
         <v>299</v>
       </c>
-      <c r="C135" s="7" t="s">
+      <c r="C136" s="7" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="136" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A136" s="5">
-        <f t="shared" si="1"/>
-        <v>128</v>
-      </c>
-      <c r="B136" s="6" t="s">
+    <row r="137" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A137" s="5">
+        <f t="shared" si="1"/>
+        <v>129</v>
+      </c>
+      <c r="B137" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="C136" s="7" t="s">
+      <c r="C137" s="7" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="137" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A137" s="5">
-        <f t="shared" si="1"/>
-        <v>129</v>
-      </c>
-      <c r="B137" s="6" t="s">
+    <row r="138" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A138" s="5">
+        <f t="shared" si="1"/>
+        <v>130</v>
+      </c>
+      <c r="B138" s="6" t="s">
         <v>376</v>
       </c>
-      <c r="C137" s="7" t="s">
+      <c r="C138" s="7" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="138" spans="1:3" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A138" s="5">
-        <f t="shared" si="1"/>
-        <v>130</v>
-      </c>
-      <c r="B138" s="6" t="s">
+    <row r="139" spans="1:3" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="5">
+        <f t="shared" si="1"/>
+        <v>131</v>
+      </c>
+      <c r="B139" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="C138" s="7" t="s">
+      <c r="C139" s="7" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="139" spans="1:3" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="5">
-        <f t="shared" si="1"/>
-        <v>131</v>
-      </c>
-      <c r="B139" s="8" t="s">
+    <row r="140" spans="1:3" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="5">
+        <f t="shared" si="1"/>
+        <v>132</v>
+      </c>
+      <c r="B140" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C139" s="9" t="s">
+      <c r="C140" s="9" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A140" s="5">
-        <f t="shared" ref="A140:A203" si="2">A139+1</f>
-        <v>132</v>
-      </c>
-      <c r="B140" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="C140" s="9" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" s="5">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="A141:A204" si="2">A140+1</f>
         <v>133</v>
       </c>
-      <c r="B141" s="10" t="s">
+      <c r="B141" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C141" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A142" s="5">
+        <f t="shared" si="2"/>
+        <v>134</v>
+      </c>
+      <c r="B142" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="C141" s="7" t="s">
+      <c r="C142" s="7" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="142" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A142" s="5">
-        <f t="shared" si="2"/>
-        <v>134</v>
-      </c>
-      <c r="B142" s="8" t="s">
+    <row r="143" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A143" s="5">
+        <f t="shared" si="2"/>
+        <v>135</v>
+      </c>
+      <c r="B143" s="8" t="s">
         <v>378</v>
       </c>
-      <c r="C142" s="9" t="s">
+      <c r="C143" s="9" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A143" s="5">
-        <f t="shared" si="2"/>
-        <v>135</v>
-      </c>
-      <c r="B143" s="8" t="s">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144" s="5">
+        <f t="shared" si="2"/>
+        <v>136</v>
+      </c>
+      <c r="B144" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C143" s="9" t="s">
+      <c r="C144" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="144" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A144" s="5">
-        <f t="shared" si="2"/>
-        <v>136</v>
-      </c>
-      <c r="B144" s="8" t="s">
+    <row r="145" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A145" s="5">
+        <f t="shared" si="2"/>
+        <v>137</v>
+      </c>
+      <c r="B145" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="C144" s="9" t="s">
+      <c r="C145" s="9" t="s">
         <v>381</v>
-      </c>
-    </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A145" s="5">
-        <f t="shared" si="2"/>
-        <v>137</v>
-      </c>
-      <c r="B145" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="C145" s="9" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
@@ -4079,34 +4130,34 @@
         <v>138</v>
       </c>
       <c r="B146" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="C146" s="9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A147" s="5">
+        <f t="shared" si="2"/>
+        <v>139</v>
+      </c>
+      <c r="B147" s="8" t="s">
         <v>515</v>
       </c>
-      <c r="C146" s="9" t="s">
+      <c r="C147" s="9" t="s">
         <v>516</v>
       </c>
     </row>
-    <row r="147" spans="1:3" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A147" s="5">
-        <f t="shared" si="2"/>
-        <v>139</v>
-      </c>
-      <c r="B147" s="8" t="s">
+    <row r="148" spans="1:3" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A148" s="5">
+        <f t="shared" si="2"/>
+        <v>140</v>
+      </c>
+      <c r="B148" s="8" t="s">
         <v>517</v>
       </c>
-      <c r="C147" s="9" t="s">
+      <c r="C148" s="9" t="s">
         <v>518</v>
-      </c>
-    </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A148" s="5">
-        <f t="shared" si="2"/>
-        <v>140</v>
-      </c>
-      <c r="B148" s="8" t="s">
-        <v>519</v>
-      </c>
-      <c r="C148" s="9" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
@@ -4115,10 +4166,10 @@
         <v>141</v>
       </c>
       <c r="B149" s="8" t="s">
-        <v>252</v>
+        <v>519</v>
       </c>
       <c r="C149" s="9" t="s">
-        <v>255</v>
+        <v>520</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
@@ -4127,10 +4178,10 @@
         <v>142</v>
       </c>
       <c r="B150" s="8" t="s">
-        <v>94</v>
+        <v>252</v>
       </c>
       <c r="C150" s="9" t="s">
-        <v>95</v>
+        <v>255</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
@@ -4139,10 +4190,10 @@
         <v>143</v>
       </c>
       <c r="B151" s="8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C151" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
@@ -4151,10 +4202,10 @@
         <v>144</v>
       </c>
       <c r="B152" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C152" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
@@ -4163,10 +4214,10 @@
         <v>145</v>
       </c>
       <c r="B153" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C153" s="9" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
@@ -4175,34 +4226,34 @@
         <v>146</v>
       </c>
       <c r="B154" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C154" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A155" s="5">
+        <f t="shared" si="2"/>
+        <v>147</v>
+      </c>
+      <c r="B155" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="C154" s="9" t="s">
+      <c r="C155" s="9" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="155" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A155" s="5">
-        <f t="shared" si="2"/>
-        <v>147</v>
-      </c>
-      <c r="B155" s="8" t="s">
+    <row r="156" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A156" s="5">
+        <f t="shared" si="2"/>
+        <v>148</v>
+      </c>
+      <c r="B156" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="C155" s="9" t="s">
+      <c r="C156" s="9" t="s">
         <v>105</v>
-      </c>
-    </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A156" s="5">
-        <f t="shared" si="2"/>
-        <v>148</v>
-      </c>
-      <c r="B156" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="C156" s="9" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
@@ -4210,11 +4261,11 @@
         <f t="shared" si="2"/>
         <v>149</v>
       </c>
-      <c r="B157" s="5" t="s">
-        <v>348</v>
-      </c>
-      <c r="C157" s="7" t="s">
-        <v>349</v>
+      <c r="B157" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C157" s="9" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
@@ -4222,119 +4273,119 @@
         <f t="shared" si="2"/>
         <v>150</v>
       </c>
-      <c r="B158" s="6" t="s">
+      <c r="B158" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="C158" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A159" s="5">
+        <f t="shared" si="2"/>
+        <v>151</v>
+      </c>
+      <c r="B159" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="C158" s="7" t="s">
+      <c r="C159" s="7" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="159" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A159" s="5">
-        <f t="shared" si="2"/>
-        <v>151</v>
-      </c>
-      <c r="B159" s="5" t="s">
+    <row r="160" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A160" s="5">
+        <f t="shared" si="2"/>
+        <v>152</v>
+      </c>
+      <c r="B160" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="C159" s="7" t="s">
+      <c r="C160" s="7" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A160" s="5">
-        <f t="shared" si="2"/>
-        <v>152</v>
-      </c>
-      <c r="B160" s="6" t="s">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A161" s="5">
+        <f t="shared" si="2"/>
+        <v>153</v>
+      </c>
+      <c r="B161" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="C160" s="7" t="s">
+      <c r="C161" s="7" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="161" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A161" s="5">
-        <f t="shared" si="2"/>
-        <v>153</v>
-      </c>
-      <c r="B161" s="6" t="s">
+    <row r="162" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A162" s="5">
+        <f t="shared" si="2"/>
+        <v>154</v>
+      </c>
+      <c r="B162" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="C161" s="7" t="s">
+      <c r="C162" s="7" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="162" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A162" s="5">
-        <f t="shared" si="2"/>
-        <v>154</v>
-      </c>
-      <c r="B162" s="5" t="s">
+    <row r="163" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="5">
+        <f t="shared" si="2"/>
+        <v>155</v>
+      </c>
+      <c r="B163" s="5" t="s">
         <v>338</v>
       </c>
-      <c r="C162" s="7" t="s">
+      <c r="C163" s="7" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A163" s="5">
-        <f t="shared" si="2"/>
-        <v>155</v>
-      </c>
-      <c r="B163" s="5" t="s">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A164" s="5">
+        <f t="shared" si="2"/>
+        <v>156</v>
+      </c>
+      <c r="B164" s="5" t="s">
         <v>433</v>
       </c>
-      <c r="C163" s="7" t="s">
+      <c r="C164" s="7" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="164" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A164" s="5">
-        <f t="shared" si="2"/>
-        <v>156</v>
-      </c>
-      <c r="B164" s="5" t="s">
+    <row r="165" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A165" s="5">
+        <f t="shared" si="2"/>
+        <v>157</v>
+      </c>
+      <c r="B165" s="5" t="s">
         <v>435</v>
       </c>
-      <c r="C164" s="7" t="s">
+      <c r="C165" s="7" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="165" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A165" s="5">
-        <f t="shared" si="2"/>
-        <v>157</v>
-      </c>
-      <c r="B165" s="5" t="s">
+    <row r="166" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A166" s="5">
+        <f t="shared" si="2"/>
+        <v>158</v>
+      </c>
+      <c r="B166" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="C165" s="7" t="s">
+      <c r="C166" s="7" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="166" spans="1:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A166" s="5">
-        <f t="shared" si="2"/>
-        <v>158</v>
-      </c>
-      <c r="B166" s="5" t="s">
+    <row r="167" spans="1:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A167" s="5">
+        <f t="shared" si="2"/>
+        <v>159</v>
+      </c>
+      <c r="B167" s="5" t="s">
         <v>352</v>
       </c>
-      <c r="C166" s="7" t="s">
+      <c r="C167" s="7" t="s">
         <v>353</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A167" s="5">
-        <f t="shared" si="2"/>
-        <v>159</v>
-      </c>
-      <c r="B167" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C167" s="7" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
@@ -4342,11 +4393,11 @@
         <f t="shared" si="2"/>
         <v>160</v>
       </c>
-      <c r="B168" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="C168" s="9" t="s">
-        <v>109</v>
+      <c r="B168" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C168" s="7" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
@@ -4355,10 +4406,10 @@
         <v>161</v>
       </c>
       <c r="B169" s="8" t="s">
-        <v>505</v>
+        <v>108</v>
       </c>
       <c r="C169" s="9" t="s">
-        <v>506</v>
+        <v>109</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
@@ -4367,10 +4418,10 @@
         <v>162</v>
       </c>
       <c r="B170" s="8" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C170" s="9" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
@@ -4379,10 +4430,10 @@
         <v>163</v>
       </c>
       <c r="B171" s="8" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="C171" s="9" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
@@ -4391,10 +4442,10 @@
         <v>164</v>
       </c>
       <c r="B172" s="8" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="C172" s="9" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
@@ -4403,10 +4454,10 @@
         <v>165</v>
       </c>
       <c r="B173" s="8" t="s">
-        <v>110</v>
+        <v>511</v>
       </c>
       <c r="C173" s="9" t="s">
-        <v>111</v>
+        <v>512</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
@@ -4415,82 +4466,82 @@
         <v>166</v>
       </c>
       <c r="B174" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C174" s="9" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A175" s="5">
+        <f t="shared" si="2"/>
+        <v>167</v>
+      </c>
+      <c r="B175" s="8" t="s">
         <v>513</v>
       </c>
-      <c r="C174" s="9" t="s">
+      <c r="C175" s="9" t="s">
         <v>514</v>
       </c>
     </row>
-    <row r="175" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A175" s="5">
-        <f t="shared" si="2"/>
+    <row r="176" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A176" s="5">
+        <f t="shared" si="2"/>
+        <v>168</v>
+      </c>
+      <c r="B176" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="C176" s="7" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A177" s="5">
+        <f t="shared" si="2"/>
+        <v>169</v>
+      </c>
+      <c r="B177" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C177" s="9" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A178" s="5">
+        <f t="shared" si="2"/>
+        <v>170</v>
+      </c>
+      <c r="B178" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C178" s="9" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A179" s="5">
+        <f t="shared" si="2"/>
+        <v>171</v>
+      </c>
+      <c r="B179" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="B175" s="6" t="s">
-        <v>312</v>
-      </c>
-      <c r="C175" s="7" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="176" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A176" s="5">
-        <f t="shared" si="2"/>
+      <c r="C179" s="7" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A180" s="5">
+        <f t="shared" si="2"/>
+        <v>172</v>
+      </c>
+      <c r="B180" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="B176" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="C176" s="9" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="177" spans="1:3" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A177" s="5">
-        <f t="shared" si="2"/>
-        <v>169</v>
-      </c>
-      <c r="B177" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="C177" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="178" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A178" s="5">
-        <f t="shared" si="2"/>
-        <v>170</v>
-      </c>
-      <c r="B178" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="C178" s="7" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="179" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A179" s="5">
-        <f t="shared" si="2"/>
+      <c r="C180" s="7" t="s">
         <v>171</v>
-      </c>
-      <c r="B179" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="C179" s="7" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A180" s="5">
-        <f t="shared" si="2"/>
-        <v>172</v>
-      </c>
-      <c r="B180" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="C180" s="9" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
@@ -4498,11 +4549,11 @@
         <f t="shared" si="2"/>
         <v>173</v>
       </c>
-      <c r="B181" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="C181" s="7" t="s">
-        <v>172</v>
+      <c r="B181" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C181" s="9" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
@@ -4511,10 +4562,10 @@
         <v>174</v>
       </c>
       <c r="B182" s="5" t="s">
-        <v>190</v>
+        <v>169</v>
       </c>
       <c r="C182" s="7" t="s">
-        <v>191</v>
+        <v>172</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
@@ -4522,11 +4573,11 @@
         <f t="shared" si="2"/>
         <v>175</v>
       </c>
-      <c r="B183" s="8" t="s">
-        <v>229</v>
-      </c>
-      <c r="C183" s="9" t="s">
-        <v>118</v>
+      <c r="B183" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C183" s="7" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
@@ -4535,10 +4586,10 @@
         <v>176</v>
       </c>
       <c r="B184" s="8" t="s">
-        <v>445</v>
+        <v>229</v>
       </c>
       <c r="C184" s="9" t="s">
-        <v>464</v>
+        <v>118</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
@@ -4547,34 +4598,34 @@
         <v>177</v>
       </c>
       <c r="B185" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C185" s="9" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A186" s="5">
+        <f t="shared" si="2"/>
+        <v>178</v>
+      </c>
+      <c r="B186" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="C185" s="9" t="s">
+      <c r="C186" s="9" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="186" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A186" s="5">
-        <f t="shared" si="2"/>
-        <v>178</v>
-      </c>
-      <c r="B186" s="8" t="s">
+    <row r="187" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A187" s="5">
+        <f t="shared" si="2"/>
+        <v>179</v>
+      </c>
+      <c r="B187" s="8" t="s">
         <v>521</v>
       </c>
-      <c r="C186" s="9" t="s">
+      <c r="C187" s="9" t="s">
         <v>522</v>
-      </c>
-    </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A187" s="5">
-        <f t="shared" si="2"/>
-        <v>179</v>
-      </c>
-      <c r="B187" s="6" t="s">
-        <v>314</v>
-      </c>
-      <c r="C187" s="7" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
@@ -4583,10 +4634,10 @@
         <v>180</v>
       </c>
       <c r="B188" s="6" t="s">
-        <v>446</v>
+        <v>314</v>
       </c>
       <c r="C188" s="7" t="s">
-        <v>465</v>
+        <v>315</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
@@ -4594,11 +4645,11 @@
         <f t="shared" si="2"/>
         <v>181</v>
       </c>
-      <c r="B189" s="5" t="s">
-        <v>192</v>
+      <c r="B189" s="6" t="s">
+        <v>446</v>
       </c>
       <c r="C189" s="7" t="s">
-        <v>193</v>
+        <v>465</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
@@ -4607,10 +4658,10 @@
         <v>182</v>
       </c>
       <c r="B190" s="5" t="s">
-        <v>226</v>
+        <v>192</v>
       </c>
       <c r="C190" s="7" t="s">
-        <v>227</v>
+        <v>193</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
@@ -4618,11 +4669,11 @@
         <f t="shared" si="2"/>
         <v>183</v>
       </c>
-      <c r="B191" s="6" t="s">
-        <v>316</v>
+      <c r="B191" s="5" t="s">
+        <v>226</v>
       </c>
       <c r="C191" s="7" t="s">
-        <v>317</v>
+        <v>227</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
@@ -4630,11 +4681,11 @@
         <f t="shared" si="2"/>
         <v>184</v>
       </c>
-      <c r="B192" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="C192" s="9" t="s">
-        <v>121</v>
+      <c r="B192" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="C192" s="7" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
@@ -4643,22 +4694,22 @@
         <v>185</v>
       </c>
       <c r="B193" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C193" s="9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A194" s="5">
+        <f t="shared" si="2"/>
+        <v>186</v>
+      </c>
+      <c r="B194" s="8" t="s">
         <v>372</v>
       </c>
-      <c r="C193" s="9" t="s">
+      <c r="C194" s="9" t="s">
         <v>373</v>
-      </c>
-    </row>
-    <row r="194" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A194" s="5">
-        <f t="shared" si="2"/>
-        <v>186</v>
-      </c>
-      <c r="B194" s="8" t="s">
-        <v>411</v>
-      </c>
-      <c r="C194" s="26" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="195" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4667,94 +4718,94 @@
         <v>187</v>
       </c>
       <c r="B195" s="8" t="s">
+        <v>411</v>
+      </c>
+      <c r="C195" s="26" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="5">
+        <f t="shared" si="2"/>
+        <v>188</v>
+      </c>
+      <c r="B196" s="8" t="s">
         <v>503</v>
       </c>
-      <c r="C195" s="26" t="s">
+      <c r="C196" s="26" t="s">
         <v>504</v>
       </c>
     </row>
-    <row r="196" spans="1:3" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A196" s="5">
-        <f t="shared" si="2"/>
-        <v>188</v>
-      </c>
-      <c r="B196" s="8" t="s">
+    <row r="197" spans="1:3" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="5">
+        <f t="shared" si="2"/>
+        <v>189</v>
+      </c>
+      <c r="B197" s="8" t="s">
         <v>367</v>
       </c>
-      <c r="C196" s="9" t="s">
+      <c r="C197" s="9" t="s">
         <v>466</v>
       </c>
     </row>
-    <row r="197" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A197" s="5">
-        <f t="shared" si="2"/>
-        <v>189</v>
-      </c>
-      <c r="B197" s="8" t="s">
+    <row r="198" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A198" s="5">
+        <f t="shared" si="2"/>
+        <v>190</v>
+      </c>
+      <c r="B198" s="8" t="s">
         <v>482</v>
       </c>
-      <c r="C197" s="9" t="s">
+      <c r="C198" s="9" t="s">
         <v>481</v>
       </c>
     </row>
-    <row r="198" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A198" s="5">
-        <f t="shared" si="2"/>
-        <v>190</v>
-      </c>
-      <c r="B198" s="8" t="s">
+    <row r="199" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A199" s="5">
+        <f t="shared" si="2"/>
+        <v>191</v>
+      </c>
+      <c r="B199" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="C198" s="9" t="s">
+      <c r="C199" s="9" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="199" spans="1:3" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A199" s="5">
-        <f t="shared" si="2"/>
-        <v>191</v>
-      </c>
-      <c r="B199" s="8" t="s">
+    <row r="200" spans="1:3" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A200" s="5">
+        <f t="shared" si="2"/>
+        <v>192</v>
+      </c>
+      <c r="B200" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="C199" s="9" t="s">
+      <c r="C200" s="9" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="200" spans="1:3" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A200" s="5">
-        <f t="shared" si="2"/>
-        <v>192</v>
-      </c>
-      <c r="B200" s="8" t="s">
+    <row r="201" spans="1:3" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A201" s="5">
+        <f t="shared" si="2"/>
+        <v>193</v>
+      </c>
+      <c r="B201" s="8" t="s">
         <v>392</v>
       </c>
-      <c r="C200" s="9" t="s">
+      <c r="C201" s="9" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="201" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A201" s="5">
-        <f t="shared" si="2"/>
-        <v>193</v>
-      </c>
-      <c r="B201" s="8" t="s">
+    <row r="202" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A202" s="5">
+        <f t="shared" si="2"/>
+        <v>194</v>
+      </c>
+      <c r="B202" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="C201" s="9" t="s">
+      <c r="C202" s="9" t="s">
         <v>126</v>
-      </c>
-    </row>
-    <row r="202" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A202" s="5">
-        <f t="shared" si="2"/>
-        <v>194</v>
-      </c>
-      <c r="B202" s="8" t="s">
-        <v>368</v>
-      </c>
-      <c r="C202" s="9" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="203" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
@@ -4762,59 +4813,59 @@
         <f t="shared" si="2"/>
         <v>195</v>
       </c>
-      <c r="B203" s="30" t="s">
+      <c r="B203" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="C203" s="9" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A204" s="5">
+        <f t="shared" si="2"/>
+        <v>196</v>
+      </c>
+      <c r="B204" s="30" t="s">
         <v>499</v>
       </c>
-      <c r="C203" s="9" t="s">
+      <c r="C204" s="9" t="s">
         <v>500</v>
-      </c>
-    </row>
-    <row r="204" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A204" s="5">
-        <f t="shared" ref="A204:A213" si="3">A203+1</f>
-        <v>196</v>
-      </c>
-      <c r="B204" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="C204" s="7" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="205" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="A205:A268" si="3">A204+1</f>
         <v>197</v>
       </c>
       <c r="B205" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="C205" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="206" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A206" s="5">
+        <f t="shared" si="3"/>
+        <v>198</v>
+      </c>
+      <c r="B206" s="5" t="s">
         <v>497</v>
       </c>
-      <c r="C205" s="7" t="s">
+      <c r="C206" s="7" t="s">
         <v>498</v>
       </c>
     </row>
-    <row r="206" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A206" s="5">
-        <f t="shared" si="3"/>
-        <v>198</v>
-      </c>
-      <c r="B206" s="5" t="s">
+    <row r="207" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A207" s="5">
+        <f t="shared" si="3"/>
+        <v>199</v>
+      </c>
+      <c r="B207" s="5" t="s">
         <v>413</v>
       </c>
-      <c r="C206" s="7" t="s">
+      <c r="C207" s="7" t="s">
         <v>416</v>
-      </c>
-    </row>
-    <row r="207" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A207" s="5">
-        <f t="shared" si="3"/>
-        <v>199</v>
-      </c>
-      <c r="B207" s="5" t="s">
-        <v>414</v>
-      </c>
-      <c r="C207" s="7" t="s">
-        <v>417</v>
       </c>
     </row>
     <row r="208" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -4823,22 +4874,22 @@
         <v>200</v>
       </c>
       <c r="B208" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="C208" s="7" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A209" s="5">
+        <f t="shared" si="3"/>
+        <v>201</v>
+      </c>
+      <c r="B209" s="5" t="s">
         <v>415</v>
       </c>
-      <c r="C208" s="7" t="s">
+      <c r="C209" s="7" t="s">
         <v>418</v>
-      </c>
-    </row>
-    <row r="209" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A209" s="5">
-        <f t="shared" si="3"/>
-        <v>201</v>
-      </c>
-      <c r="B209" s="32" t="s">
-        <v>530</v>
-      </c>
-      <c r="C209" s="33" t="s">
-        <v>531</v>
       </c>
     </row>
     <row r="210" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -4847,10 +4898,10 @@
         <v>202</v>
       </c>
       <c r="B210" s="32" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="C210" s="33" t="s">
-        <v>535</v>
+        <v>531</v>
       </c>
     </row>
     <row r="211" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -4859,10 +4910,10 @@
         <v>203</v>
       </c>
       <c r="B211" s="32" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="C211" s="33" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
     </row>
     <row r="212" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -4871,10 +4922,10 @@
         <v>204</v>
       </c>
       <c r="B212" s="32" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C212" s="33" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="213" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -4883,841 +4934,931 @@
         <v>205</v>
       </c>
       <c r="B213" s="32" t="s">
-        <v>539</v>
+        <v>534</v>
       </c>
       <c r="C213" s="33" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="214" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A214" s="5">
+        <f t="shared" si="3"/>
         <v>206</v>
       </c>
-      <c r="B214" s="5" t="s">
+      <c r="B214" s="32" t="s">
+        <v>539</v>
+      </c>
+      <c r="C214" s="33" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A215" s="5">
+        <f t="shared" si="3"/>
+        <v>207</v>
+      </c>
+      <c r="B215" s="5" t="s">
         <v>550</v>
       </c>
-      <c r="C214" s="42" t="s">
+      <c r="C215" s="41" t="s">
         <v>551</v>
-      </c>
-    </row>
-    <row r="215" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A215" s="5">
-        <v>207</v>
-      </c>
-      <c r="B215" s="5" t="s">
-        <v>552</v>
-      </c>
-      <c r="C215" s="7" t="s">
-        <v>553</v>
       </c>
     </row>
     <row r="216" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A216" s="5">
+        <f t="shared" si="3"/>
         <v>208</v>
       </c>
       <c r="B216" s="5" t="s">
+        <v>552</v>
+      </c>
+      <c r="C216" s="7" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A217" s="5">
+        <f t="shared" si="3"/>
+        <v>209</v>
+      </c>
+      <c r="B217" s="5" t="s">
         <v>419</v>
       </c>
-      <c r="C216" s="7" t="s">
+      <c r="C217" s="7" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="217" spans="1:3" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A217" s="5">
-        <v>209</v>
-      </c>
-      <c r="B217" s="24" t="s">
+    <row r="218" spans="1:3" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A218" s="5">
+        <f t="shared" si="3"/>
+        <v>210</v>
+      </c>
+      <c r="B218" s="24" t="s">
         <v>455</v>
       </c>
-      <c r="C217" s="9" t="s">
+      <c r="C218" s="9" t="s">
         <v>456</v>
       </c>
     </row>
-    <row r="218" spans="1:3" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A218" s="5">
-        <v>210</v>
-      </c>
-      <c r="B218" s="24" t="s">
+    <row r="219" spans="1:3" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A219" s="5">
+        <f t="shared" si="3"/>
+        <v>211</v>
+      </c>
+      <c r="B219" s="24" t="s">
         <v>523</v>
       </c>
-      <c r="C218" s="9" t="s">
+      <c r="C219" s="9" t="s">
         <v>524</v>
       </c>
     </row>
-    <row r="219" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A219" s="5">
-        <v>211</v>
-      </c>
-      <c r="B219" s="5" t="s">
+    <row r="220" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A220" s="5">
+        <f t="shared" si="3"/>
+        <v>212</v>
+      </c>
+      <c r="B220" s="5" t="s">
         <v>554</v>
       </c>
-      <c r="C219" s="7" t="s">
+      <c r="C220" s="7" t="s">
         <v>555</v>
-      </c>
-    </row>
-    <row r="220" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A220" s="5">
-        <v>212</v>
-      </c>
-      <c r="B220" s="5" t="s">
-        <v>421</v>
-      </c>
-      <c r="C220" s="7" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="221" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A221" s="5">
+        <f t="shared" si="3"/>
         <v>213</v>
       </c>
       <c r="B221" s="5" t="s">
+        <v>421</v>
+      </c>
+      <c r="C221" s="7" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A222" s="5">
+        <f t="shared" si="3"/>
+        <v>214</v>
+      </c>
+      <c r="B222" s="5" t="s">
         <v>525</v>
       </c>
-      <c r="C221" s="7" t="s">
+      <c r="C222" s="7" t="s">
         <v>526</v>
       </c>
     </row>
-    <row r="222" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A222" s="5">
-        <v>214</v>
-      </c>
-      <c r="B222" s="5" t="s">
+    <row r="223" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A223" s="5">
+        <f t="shared" si="3"/>
+        <v>215</v>
+      </c>
+      <c r="B223" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="C222" s="7" t="s">
+      <c r="C223" s="7" t="s">
         <v>189</v>
-      </c>
-    </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A223" s="5">
-        <v>215</v>
-      </c>
-      <c r="B223" s="5" t="s">
-        <v>333</v>
-      </c>
-      <c r="C223" s="7" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" s="5">
+        <f t="shared" si="3"/>
         <v>216</v>
       </c>
-      <c r="B224" s="6" t="s">
-        <v>318</v>
+      <c r="B224" s="5" t="s">
+        <v>333</v>
       </c>
       <c r="C224" s="7" t="s">
-        <v>319</v>
+        <v>334</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" s="5">
+        <f t="shared" si="3"/>
         <v>217</v>
       </c>
       <c r="B225" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="C225" s="7" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A226" s="5">
+        <f t="shared" si="3"/>
+        <v>218</v>
+      </c>
+      <c r="B226" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="C225" s="7" t="s">
+      <c r="C226" s="7" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="226" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A226" s="5">
-        <v>218</v>
-      </c>
-      <c r="B226" s="8" t="s">
+    <row r="227" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A227" s="5">
+        <f t="shared" si="3"/>
+        <v>219</v>
+      </c>
+      <c r="B227" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="C226" s="9" t="s">
+      <c r="C227" s="9" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A227" s="5">
-        <v>219</v>
-      </c>
-      <c r="B227" s="6" t="s">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A228" s="5">
+        <f t="shared" si="3"/>
+        <v>220</v>
+      </c>
+      <c r="B228" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="C227" s="7" t="s">
+      <c r="C228" s="7" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="228" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A228" s="5">
-        <v>220</v>
-      </c>
-      <c r="B228" s="6" t="s">
+    <row r="229" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A229" s="5">
+        <f t="shared" si="3"/>
+        <v>221</v>
+      </c>
+      <c r="B229" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="C228" s="7" t="s">
+      <c r="C229" s="7" t="s">
         <v>325</v>
-      </c>
-    </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A229" s="5">
-        <v>221</v>
-      </c>
-      <c r="B229" s="6" t="s">
-        <v>326</v>
-      </c>
-      <c r="C229" s="7" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" s="5">
+        <f t="shared" si="3"/>
         <v>222</v>
       </c>
       <c r="B230" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C230" s="7" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A231" s="5">
+        <f t="shared" si="3"/>
+        <v>223</v>
+      </c>
+      <c r="B231" s="6" t="s">
         <v>328</v>
       </c>
-      <c r="C230" s="7" t="s">
+      <c r="C231" s="7" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="231" spans="1:3" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A231" s="5">
-        <v>223</v>
-      </c>
-      <c r="B231" s="5" t="s">
+    <row r="232" spans="1:3" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A232" s="5">
+        <f t="shared" si="3"/>
+        <v>224</v>
+      </c>
+      <c r="B232" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="C231" s="7" t="s">
+      <c r="C232" s="7" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="232" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A232" s="5">
-        <v>224</v>
-      </c>
-      <c r="B232" s="5" t="s">
+    <row r="233" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A233" s="5">
+        <f t="shared" si="3"/>
+        <v>225</v>
+      </c>
+      <c r="B233" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C232" s="7" t="s">
+      <c r="C233" s="7" t="s">
         <v>9</v>
-      </c>
-    </row>
-    <row r="233" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A233" s="5">
-        <v>225</v>
-      </c>
-      <c r="B233" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="C233" s="7" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="234" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A234" s="5">
+        <f t="shared" si="3"/>
         <v>226</v>
       </c>
       <c r="B234" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="C234" s="7" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A235" s="5">
+        <f t="shared" si="3"/>
+        <v>227</v>
+      </c>
+      <c r="B235" s="5" t="s">
         <v>387</v>
       </c>
-      <c r="C234" s="7" t="s">
+      <c r="C235" s="7" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="235" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A235" s="5">
-        <v>227</v>
-      </c>
-      <c r="B235" s="5" t="s">
+    <row r="236" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A236" s="5">
+        <f t="shared" si="3"/>
+        <v>228</v>
+      </c>
+      <c r="B236" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="C235" s="7" t="s">
+      <c r="C236" s="7" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="236" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A236" s="5">
-        <v>228</v>
-      </c>
-      <c r="B236" s="5" t="s">
+    <row r="237" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A237" s="5">
+        <f t="shared" si="3"/>
+        <v>229</v>
+      </c>
+      <c r="B237" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="C236" s="7" t="s">
+      <c r="C237" s="7" t="s">
         <v>164</v>
-      </c>
-    </row>
-    <row r="237" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A237" s="5">
-        <v>229</v>
-      </c>
-      <c r="B237" s="8" t="s">
-        <v>382</v>
-      </c>
-      <c r="C237" s="7" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="238" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A238" s="5">
+        <f t="shared" si="3"/>
         <v>230</v>
       </c>
-      <c r="B238" s="5" t="s">
-        <v>198</v>
+      <c r="B238" s="8" t="s">
+        <v>382</v>
       </c>
       <c r="C238" s="7" t="s">
-        <v>199</v>
+        <v>383</v>
       </c>
     </row>
     <row r="239" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A239" s="5">
+        <f t="shared" si="3"/>
         <v>231</v>
       </c>
       <c r="B239" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C239" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A240" s="5">
+        <f t="shared" si="3"/>
+        <v>232</v>
+      </c>
+      <c r="B240" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="C239" s="7" t="s">
+      <c r="C240" s="7" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="240" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A240" s="5">
-        <v>232</v>
-      </c>
-      <c r="B240" s="8" t="s">
+    <row r="241" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A241" s="5">
+        <f t="shared" si="3"/>
+        <v>233</v>
+      </c>
+      <c r="B241" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="C240" s="7" t="s">
+      <c r="C241" s="7" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="241" spans="1:3" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A241" s="5">
-        <v>233</v>
-      </c>
-      <c r="B241" s="8" t="s">
+    <row r="242" spans="1:3" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A242" s="5">
+        <f t="shared" si="3"/>
+        <v>234</v>
+      </c>
+      <c r="B242" s="8" t="s">
         <v>384</v>
       </c>
-      <c r="C241" s="7" t="s">
+      <c r="C242" s="7" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="242" spans="1:3" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A242" s="5">
-        <v>234</v>
-      </c>
-      <c r="B242" s="8" t="s">
+    <row r="243" spans="1:3" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A243" s="5">
+        <f t="shared" si="3"/>
+        <v>235</v>
+      </c>
+      <c r="B243" s="8" t="s">
         <v>360</v>
       </c>
-      <c r="C242" s="7" t="s">
+      <c r="C243" s="7" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="243" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A243" s="5">
-        <v>235</v>
-      </c>
-      <c r="B243" s="8" t="s">
+    <row r="244" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A244" s="5">
+        <f t="shared" si="3"/>
+        <v>236</v>
+      </c>
+      <c r="B244" s="8" t="s">
         <v>409</v>
       </c>
-      <c r="C243" s="7" t="s">
+      <c r="C244" s="7" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="244" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A244" s="5">
-        <v>236</v>
-      </c>
-      <c r="B244" s="8" t="s">
+    <row r="245" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A245" s="5">
+        <f t="shared" si="3"/>
+        <v>237</v>
+      </c>
+      <c r="B245" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C244" s="7" t="s">
+      <c r="C245" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="245" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A245" s="5">
-        <v>237</v>
-      </c>
-      <c r="B245" s="8" t="s">
+    <row r="246" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A246" s="5">
+        <f t="shared" si="3"/>
+        <v>238</v>
+      </c>
+      <c r="B246" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C245" s="7" t="s">
+      <c r="C246" s="7" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="246" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A246" s="5">
-        <v>238</v>
-      </c>
-      <c r="B246" s="5" t="s">
+    <row r="247" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A247" s="5">
+        <f t="shared" si="3"/>
+        <v>239</v>
+      </c>
+      <c r="B247" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C246" s="7" t="s">
+      <c r="C247" s="7" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A247" s="5">
-        <v>239</v>
-      </c>
-      <c r="B247" s="5" t="s">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A248" s="5">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+      <c r="B248" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="C247" s="7" t="s">
+      <c r="C248" s="7" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="248" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A248" s="5">
-        <v>240</v>
-      </c>
-      <c r="B248" s="5" t="s">
+    <row r="249" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A249" s="5">
+        <f t="shared" si="3"/>
+        <v>241</v>
+      </c>
+      <c r="B249" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="C248" s="7" t="s">
+      <c r="C249" s="7" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="249" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A249" s="5">
-        <v>241</v>
-      </c>
-      <c r="B249" s="5" t="s">
+    <row r="250" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A250" s="5">
+        <f t="shared" si="3"/>
+        <v>242</v>
+      </c>
+      <c r="B250" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="C249" s="7" t="s">
+      <c r="C250" s="7" t="s">
         <v>247</v>
-      </c>
-    </row>
-    <row r="250" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A250" s="5">
-        <v>242</v>
-      </c>
-      <c r="B250" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C250" s="7" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="251" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A251" s="5">
+        <f t="shared" si="3"/>
         <v>243</v>
       </c>
       <c r="B251" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C251" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="252" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A252" s="5">
+        <f t="shared" si="3"/>
+        <v>244</v>
+      </c>
+      <c r="B252" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C251" s="7" t="s">
+      <c r="C252" s="7" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A252" s="5">
-        <v>244</v>
-      </c>
-      <c r="B252" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="C252" s="7" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" s="5">
+        <f t="shared" si="3"/>
         <v>245</v>
       </c>
       <c r="B253" s="8" t="s">
-        <v>386</v>
+        <v>233</v>
       </c>
       <c r="C253" s="7" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" s="5">
+        <f t="shared" si="3"/>
         <v>246</v>
       </c>
       <c r="B254" s="8" t="s">
-        <v>236</v>
+        <v>386</v>
       </c>
       <c r="C254" s="7" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="255" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" s="5">
+        <f t="shared" si="3"/>
         <v>247</v>
       </c>
       <c r="B255" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="C255" s="7" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="256" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A256" s="5">
+        <f t="shared" si="3"/>
+        <v>248</v>
+      </c>
+      <c r="B256" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="C255" s="9" t="s">
+      <c r="C256" s="9" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="256" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A256" s="5">
-        <v>248</v>
-      </c>
-      <c r="B256" s="8" t="s">
+    <row r="257" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A257" s="5">
+        <f t="shared" si="3"/>
+        <v>249</v>
+      </c>
+      <c r="B257" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="C256" s="9" t="s">
+      <c r="C257" s="9" t="s">
         <v>132</v>
-      </c>
-    </row>
-    <row r="257" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A257" s="5">
-        <v>249</v>
-      </c>
-      <c r="B257" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="C257" s="9" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="258" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A258" s="5">
+        <f t="shared" si="3"/>
         <v>250</v>
       </c>
       <c r="B258" s="8" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C258" s="9" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="259" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A259" s="5">
+        <f t="shared" si="3"/>
         <v>251</v>
       </c>
-      <c r="B259" s="5" t="s">
+      <c r="B259" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="C259" s="9" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="260" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A260" s="5">
+        <f t="shared" si="3"/>
+        <v>252</v>
+      </c>
+      <c r="B260" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="C259" s="9" t="s">
+      <c r="C260" s="9" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A260" s="5">
-        <v>252</v>
-      </c>
-      <c r="B260" s="8" t="s">
+    <row r="261" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A261" s="5">
+        <f t="shared" si="3"/>
+        <v>253</v>
+      </c>
+      <c r="B261" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="C260" s="9" t="s">
+      <c r="C261" s="9" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="261" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A261" s="5">
-        <v>253</v>
-      </c>
-      <c r="B261" s="8" t="s">
+    <row r="262" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A262" s="5">
+        <f t="shared" si="3"/>
+        <v>254</v>
+      </c>
+      <c r="B262" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="C261" s="9" t="s">
+      <c r="C262" s="9" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A262" s="5">
-        <v>254</v>
-      </c>
-      <c r="B262" s="8" t="s">
+    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A263" s="5">
+        <f t="shared" si="3"/>
+        <v>255</v>
+      </c>
+      <c r="B263" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="C262" s="9" t="s">
+      <c r="C263" s="9" t="s">
         <v>144</v>
-      </c>
-    </row>
-    <row r="263" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A263" s="5">
-        <v>255</v>
-      </c>
-      <c r="B263" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="C263" s="7" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="264" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A264" s="5">
+        <f t="shared" si="3"/>
         <v>256</v>
       </c>
       <c r="B264" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C264" s="7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A265" s="5">
+        <f t="shared" si="3"/>
+        <v>257</v>
+      </c>
+      <c r="B265" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="C264" s="7" t="s">
+      <c r="C265" s="7" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A265" s="5">
-        <v>257</v>
-      </c>
-      <c r="B265" s="31" t="s">
+    <row r="266" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A266" s="5">
+        <f t="shared" si="3"/>
+        <v>258</v>
+      </c>
+      <c r="B266" s="31" t="s">
         <v>527</v>
       </c>
-      <c r="C265" s="7" t="s">
+      <c r="C266" s="7" t="s">
         <v>528</v>
       </c>
     </row>
-    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A266" s="5">
-        <v>258</v>
-      </c>
-      <c r="B266" s="8" t="s">
+    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A267" s="5">
+        <f t="shared" si="3"/>
+        <v>259</v>
+      </c>
+      <c r="B267" s="8" t="s">
         <v>354</v>
       </c>
-      <c r="C266" s="7" t="s">
+      <c r="C267" s="7" t="s">
         <v>355</v>
-      </c>
-    </row>
-    <row r="267" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A267" s="5">
-        <v>259</v>
-      </c>
-      <c r="B267" s="8" t="s">
-        <v>250</v>
-      </c>
-      <c r="C267" s="7" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="268" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A268" s="5">
+        <f t="shared" si="3"/>
         <v>260</v>
       </c>
       <c r="B268" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C268" s="7" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="269" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A269" s="5">
+        <f t="shared" ref="A269:A288" si="4">A268+1</f>
+        <v>261</v>
+      </c>
+      <c r="B269" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C268" s="7" t="s">
+      <c r="C269" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="269" spans="1:3" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A269" s="24">
-        <v>261</v>
-      </c>
-      <c r="B269" s="41" t="s">
+    <row r="270" spans="1:3" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A270" s="5">
+        <f t="shared" si="4"/>
+        <v>262</v>
+      </c>
+      <c r="B270" s="40" t="s">
         <v>558</v>
       </c>
-      <c r="C269" s="9" t="s">
+      <c r="C270" s="9" t="s">
         <v>559</v>
       </c>
     </row>
-    <row r="270" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A270" s="5">
-        <v>262</v>
-      </c>
-      <c r="B270" s="8" t="s">
+    <row r="271" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A271" s="5">
+        <f t="shared" si="4"/>
+        <v>263</v>
+      </c>
+      <c r="B271" s="8" t="s">
         <v>356</v>
       </c>
-      <c r="C270" s="7" t="s">
+      <c r="C271" s="7" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="271" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A271" s="5">
-        <v>263</v>
-      </c>
-      <c r="B271" s="8" t="s">
+    <row r="272" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A272" s="5">
+        <f t="shared" si="4"/>
+        <v>264</v>
+      </c>
+      <c r="B272" s="8" t="s">
         <v>453</v>
       </c>
-      <c r="C271" s="7" t="s">
+      <c r="C272" s="7" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="272" spans="1:3" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A272" s="5">
-        <v>264</v>
-      </c>
-      <c r="B272" s="8" t="s">
+    <row r="273" spans="1:10" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A273" s="5">
+        <f t="shared" si="4"/>
+        <v>265</v>
+      </c>
+      <c r="B273" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C272" s="7" t="s">
+      <c r="C273" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="273" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A273" s="5">
-        <v>265</v>
-      </c>
-      <c r="B273" s="29" t="s">
+    <row r="274" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A274" s="5">
+        <f t="shared" si="4"/>
+        <v>266</v>
+      </c>
+      <c r="B274" s="29" t="s">
         <v>489</v>
       </c>
-      <c r="C273" s="28" t="s">
+      <c r="C274" s="28" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="274" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A274" s="5">
-        <v>266</v>
-      </c>
-      <c r="B274" s="8" t="s">
+    <row r="275" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A275" s="5">
+        <f t="shared" si="4"/>
+        <v>267</v>
+      </c>
+      <c r="B275" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C274" s="7" t="s">
+      <c r="C275" s="7" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="275" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A275" s="5">
-        <v>267</v>
-      </c>
-      <c r="B275" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="C275" s="7" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="276" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A276" s="5">
+        <f t="shared" si="4"/>
         <v>268</v>
       </c>
-      <c r="B276" s="6" t="s">
-        <v>330</v>
+      <c r="B276" s="5" t="s">
+        <v>150</v>
       </c>
       <c r="C276" s="7" t="s">
-        <v>331</v>
+        <v>151</v>
       </c>
     </row>
     <row r="277" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A277" s="5">
+        <f t="shared" si="4"/>
         <v>269</v>
       </c>
-      <c r="B277" s="5" t="s">
-        <v>230</v>
+      <c r="B277" s="6" t="s">
+        <v>330</v>
       </c>
       <c r="C277" s="7" t="s">
-        <v>231</v>
+        <v>331</v>
       </c>
     </row>
     <row r="278" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A278" s="5">
+        <f t="shared" si="4"/>
         <v>270</v>
       </c>
       <c r="B278" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="C278" s="7" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="279" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A279" s="5">
+        <f t="shared" si="4"/>
+        <v>271</v>
+      </c>
+      <c r="B279" s="5" t="s">
         <v>423</v>
       </c>
-      <c r="C278" s="7" t="s">
+      <c r="C279" s="7" t="s">
         <v>424</v>
       </c>
-      <c r="J278" s="21"/>
-    </row>
-    <row r="279" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A279" s="5">
-        <v>271</v>
-      </c>
-      <c r="B279" s="5" t="s">
+      <c r="J279" s="21"/>
+    </row>
+    <row r="280" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A280" s="5">
+        <f t="shared" si="4"/>
+        <v>272</v>
+      </c>
+      <c r="B280" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="C279" s="7" t="s">
+      <c r="C280" s="7" t="s">
         <v>238</v>
-      </c>
-    </row>
-    <row r="280" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A280" s="5">
-        <v>272</v>
-      </c>
-      <c r="B280" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="C280" s="7" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="281" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A281" s="5">
+        <f t="shared" si="4"/>
         <v>273</v>
       </c>
       <c r="B281" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="C281" s="7" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="282" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A282" s="5">
+        <f t="shared" si="4"/>
+        <v>274</v>
+      </c>
+      <c r="B282" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C281" s="7" t="s">
+      <c r="C282" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="282" spans="1:10" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A282" s="5">
-        <v>274</v>
-      </c>
-      <c r="B282" s="5" t="s">
+    <row r="283" spans="1:10" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A283" s="5">
+        <f t="shared" si="4"/>
+        <v>275</v>
+      </c>
+      <c r="B283" s="5" t="s">
         <v>437</v>
       </c>
-      <c r="C282" s="22" t="s">
+      <c r="C283" s="22" t="s">
         <v>438</v>
       </c>
     </row>
-    <row r="283" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A283" s="5">
-        <v>275</v>
-      </c>
-      <c r="B283" s="5" t="s">
+    <row r="284" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A284" s="5">
+        <f t="shared" si="4"/>
+        <v>276</v>
+      </c>
+      <c r="B284" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="C283" s="7" t="s">
+      <c r="C284" s="7" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="284" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A284" s="5">
-        <v>276</v>
-      </c>
-      <c r="B284" s="5" t="s">
+    <row r="285" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A285" s="5">
+        <f t="shared" si="4"/>
+        <v>277</v>
+      </c>
+      <c r="B285" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="C284" s="23" t="s">
+      <c r="C285" s="23" t="s">
         <v>557</v>
       </c>
     </row>
-    <row r="285" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A285" s="5">
-        <v>277</v>
-      </c>
-      <c r="B285" s="43" t="s">
+    <row r="286" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A286" s="5">
+        <f t="shared" si="4"/>
+        <v>278</v>
+      </c>
+      <c r="B286" s="42" t="s">
         <v>560</v>
       </c>
-      <c r="C285" s="45" t="s">
+      <c r="C286" s="44" t="s">
         <v>561</v>
       </c>
     </row>
-    <row r="286" spans="1:10" s="25" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A286" s="5">
-        <v>278</v>
-      </c>
-      <c r="B286" s="44" t="s">
+    <row r="287" spans="1:10" s="25" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A287" s="5">
+        <f t="shared" si="4"/>
+        <v>279</v>
+      </c>
+      <c r="B287" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="C286" s="7" t="s">
+      <c r="C287" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="287" spans="1:10" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A287" s="5">
-        <v>279</v>
-      </c>
-      <c r="B287" s="5" t="s">
+    <row r="288" spans="1:10" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A288" s="5">
+        <f t="shared" si="4"/>
+        <v>280</v>
+      </c>
+      <c r="B288" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="C287" s="7" t="s">
+      <c r="C288" s="7" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="288" spans="1:10" ht="15" x14ac:dyDescent="0.25">
-      <c r="A288" s="1"/>
-      <c r="B288" s="1"/>
-      <c r="C288" s="1"/>
-    </row>
-    <row r="290" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C290" s="40"/>
-      <c r="D290" s="36"/>
-      <c r="E290" s="37"/>
-      <c r="F290" s="37"/>
-      <c r="G290" s="38"/>
-      <c r="H290" s="12"/>
-      <c r="I290" s="12"/>
-      <c r="J290" s="12"/>
+    <row r="289" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="A289" s="1"/>
+      <c r="B289" s="1"/>
+      <c r="C289" s="1"/>
+    </row>
+    <row r="291" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A291" s="46"/>
+      <c r="B291" s="45"/>
+      <c r="C291" s="46" t="s">
+        <v>565</v>
+      </c>
+      <c r="D291" s="36"/>
+      <c r="E291" s="37"/>
+      <c r="F291" s="37"/>
+      <c r="G291" s="38"/>
+      <c r="H291" s="12"/>
+      <c r="I291" s="12"/>
+      <c r="J291" s="12"/>
     </row>
   </sheetData>
   <autoFilter ref="A8:C8" xr:uid="{00000000-0009-0000-0000-000000000000}">
@@ -5729,7 +5870,7 @@
     <mergeCell ref="A5:C7"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="66" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="63" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>